<commit_message>
WIP: 2026-10-08 team posts in progress
</commit_message>
<xml_diff>
--- a/templates/tidy-tabs-remove-non-breaking-spaces.xlsx
+++ b/templates/tidy-tabs-remove-non-breaking-spaces.xlsx
@@ -542,7 +542,7 @@
         <v/>
       </c>
       <c r="C2" s="3">
-        <f>CODE(MID(A2,5,1))</f>
+        <f>_xlfn.UNICODE(MID(A2,5,1))</f>
         <v/>
       </c>
       <c r="D2" s="3">
@@ -550,7 +550,7 @@
         <v/>
       </c>
       <c r="E2" s="3">
-        <f>TRIM(CLEAN(SUBSTITUTE(A2,CHAR(160)," ")))</f>
+        <f>TRIM(CLEAN(SUBSTITUTE(A2,_xlfn.UNICHAR(160)," ")))</f>
         <v/>
       </c>
       <c r="F2" s="3">
@@ -593,7 +593,7 @@
         <v/>
       </c>
       <c r="C3" s="3">
-        <f>CODE(MID(A3,5,1))</f>
+        <f>_xlfn.UNICODE(MID(A3,5,1))</f>
         <v/>
       </c>
       <c r="D3" s="3">
@@ -601,7 +601,7 @@
         <v/>
       </c>
       <c r="E3" s="3">
-        <f>TRIM(CLEAN(SUBSTITUTE(A3,CHAR(160)," ")))</f>
+        <f>TRIM(CLEAN(SUBSTITUTE(A3,_xlfn.UNICHAR(160)," ")))</f>
         <v/>
       </c>
       <c r="F3" s="3">
@@ -644,7 +644,7 @@
         <v/>
       </c>
       <c r="C4" s="3">
-        <f>CODE(MID(A4,5,1))</f>
+        <f>_xlfn.UNICODE(MID(A4,5,1))</f>
         <v/>
       </c>
       <c r="D4" s="3">
@@ -652,7 +652,7 @@
         <v/>
       </c>
       <c r="E4" s="3">
-        <f>TRIM(CLEAN(SUBSTITUTE(A4,CHAR(160)," ")))</f>
+        <f>TRIM(CLEAN(SUBSTITUTE(A4,_xlfn.UNICHAR(160)," ")))</f>
         <v/>
       </c>
       <c r="F4" s="3">
@@ -696,7 +696,7 @@
         <v/>
       </c>
       <c r="C5" s="3">
-        <f>CODE(MID(A5,5,1))</f>
+        <f>_xlfn.UNICODE(MID(A5,5,1))</f>
         <v/>
       </c>
       <c r="D5" s="3">
@@ -704,7 +704,7 @@
         <v/>
       </c>
       <c r="E5" s="3">
-        <f>TRIM(CLEAN(SUBSTITUTE(A5,CHAR(160)," ")))</f>
+        <f>TRIM(CLEAN(SUBSTITUTE(A5,_xlfn.UNICHAR(160)," ")))</f>
         <v/>
       </c>
       <c r="F5" s="3">
@@ -747,7 +747,7 @@
         <v/>
       </c>
       <c r="C6" s="3">
-        <f>CODE(MID(A6,5,1))</f>
+        <f>_xlfn.UNICODE(MID(A6,5,1))</f>
         <v/>
       </c>
       <c r="D6" s="3">
@@ -755,7 +755,7 @@
         <v/>
       </c>
       <c r="E6" s="3">
-        <f>TRIM(CLEAN(SUBSTITUTE(A6,CHAR(160)," ")))</f>
+        <f>TRIM(CLEAN(SUBSTITUTE(A6,_xlfn.UNICHAR(160)," ")))</f>
         <v/>
       </c>
       <c r="F6" s="3">
@@ -798,7 +798,7 @@
         <v/>
       </c>
       <c r="C7" s="3">
-        <f>CODE(MID(A7,5,1))</f>
+        <f>_xlfn.UNICODE(MID(A7,5,1))</f>
         <v/>
       </c>
       <c r="D7" s="3">
@@ -806,7 +806,7 @@
         <v/>
       </c>
       <c r="E7" s="3">
-        <f>TRIM(CLEAN(SUBSTITUTE(A7,CHAR(160)," ")))</f>
+        <f>TRIM(CLEAN(SUBSTITUTE(A7,_xlfn.UNICHAR(160)," ")))</f>
         <v/>
       </c>
       <c r="F7" s="3">
@@ -849,7 +849,7 @@
         <v/>
       </c>
       <c r="C8" s="3">
-        <f>CODE(MID(A8,5,1))</f>
+        <f>_xlfn.UNICODE(MID(A8,5,1))</f>
         <v/>
       </c>
       <c r="D8" s="3">
@@ -857,7 +857,7 @@
         <v/>
       </c>
       <c r="E8" s="3">
-        <f>TRIM(CLEAN(SUBSTITUTE(A8,CHAR(160)," ")))</f>
+        <f>TRIM(CLEAN(SUBSTITUTE(A8,_xlfn.UNICHAR(160)," ")))</f>
         <v/>
       </c>
       <c r="F8" s="3">
@@ -900,7 +900,7 @@
         <v/>
       </c>
       <c r="C9" s="3">
-        <f>CODE(MID(A9,5,1))</f>
+        <f>_xlfn.UNICODE(MID(A9,5,1))</f>
         <v/>
       </c>
       <c r="D9" s="3">
@@ -908,7 +908,7 @@
         <v/>
       </c>
       <c r="E9" s="3">
-        <f>TRIM(CLEAN(SUBSTITUTE(A9,CHAR(160)," ")))</f>
+        <f>TRIM(CLEAN(SUBSTITUTE(A9,_xlfn.UNICHAR(160)," ")))</f>
         <v/>
       </c>
       <c r="F9" s="3">
@@ -1006,7 +1006,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3. Column C: =CODE(MID(A2,5,1)) shows the character code at position 5. A normal space is 32, a non-breaking space is 160. This works here because every first name has 4 letters; change the 5 to point at the character you suspect.</t>
+          <t>3. Column C: =UNICODE(MID(A2,5,1)) shows the character code at position 5 (=CODE(MID(A2,5,1)) is the older version, but in LibreOffice it returned 160 in one setup and 194 in another, depending on the locale). A normal space is 32, a non-breaking space is 160. This works here because every first name has 4 letters; change the 5 to point at the character you suspect.</t>
         </is>
       </c>
     </row>
@@ -1020,7 +1020,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>5. Column E: =TRIM(CLEAN(SUBSTITUTE(A2,CHAR(160)," "))). SUBSTITUTE swaps character 160 for a normal space, CLEAN removes line breaks and tabs, TRIM removes extra spaces.</t>
+          <t>5. Column E: =TRIM(CLEAN(SUBSTITUTE(A2,UNICHAR(160)," "))). UNICHAR(160) is used instead of CHAR(160) because LibreOffice returned a different character for CHAR(160) in one setup. SUBSTITUTE swaps character 160 for a normal space, CLEAN removes line breaks and tabs, TRIM removes extra spaces.</t>
         </is>
       </c>
     </row>

</xml_diff>